<commit_message>
unify etapa and forecast bot
</commit_message>
<xml_diff>
--- a/ferniq_oportunidad_scraper/resultado_etapa_ferniq.xlsx
+++ b/ferniq_oportunidad_scraper/resultado_etapa_ferniq.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detalle" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Resumen" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Detalle" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -832,7 +832,7 @@
       </c>
       <c r="G2" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22 09:51:21</t>
+          <t>2026-05-26 00:21:27</t>
         </is>
       </c>
       <c r="H2" s="1" t="inlineStr">
@@ -868,7 +868,7 @@
       </c>
       <c r="G3" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22 09:51:21</t>
+          <t>2026-05-26 00:21:27</t>
         </is>
       </c>
       <c r="H3" s="1" t="inlineStr">
@@ -904,7 +904,7 @@
       </c>
       <c r="G4" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22 09:51:21</t>
+          <t>2026-05-26 00:21:27</t>
         </is>
       </c>
       <c r="H4" s="1" t="inlineStr">
@@ -940,7 +940,7 @@
       </c>
       <c r="G5" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22 09:51:21</t>
+          <t>2026-05-26 00:21:27</t>
         </is>
       </c>
       <c r="H5" s="1" t="inlineStr">
@@ -976,7 +976,7 @@
       </c>
       <c r="G6" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22 09:51:21</t>
+          <t>2026-05-26 00:21:27</t>
         </is>
       </c>
       <c r="H6" s="1" t="inlineStr">
@@ -1012,7 +1012,7 @@
       </c>
       <c r="G7" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22 09:51:21</t>
+          <t>2026-05-26 00:21:27</t>
         </is>
       </c>
       <c r="H7" s="1" t="inlineStr">
@@ -1048,7 +1048,7 @@
       </c>
       <c r="G8" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22 09:51:21</t>
+          <t>2026-05-26 00:21:27</t>
         </is>
       </c>
       <c r="H8" s="1" t="inlineStr">
@@ -1084,7 +1084,7 @@
       </c>
       <c r="G9" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22 09:51:21</t>
+          <t>2026-05-26 00:21:27</t>
         </is>
       </c>
       <c r="H9" s="1" t="inlineStr">
@@ -1120,7 +1120,7 @@
       </c>
       <c r="G10" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22 09:51:21</t>
+          <t>2026-05-26 00:21:27</t>
         </is>
       </c>
       <c r="H10" s="1" t="inlineStr">
@@ -1156,7 +1156,7 @@
       </c>
       <c r="G11" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22 09:51:21</t>
+          <t>2026-05-26 00:21:27</t>
         </is>
       </c>
       <c r="H11" s="1" t="inlineStr">
@@ -1192,7 +1192,7 @@
       </c>
       <c r="G12" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22 09:51:21</t>
+          <t>2026-05-26 00:21:27</t>
         </is>
       </c>
       <c r="H12" s="1" t="inlineStr">
@@ -1228,7 +1228,7 @@
       </c>
       <c r="G13" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22 09:51:21</t>
+          <t>2026-05-26 00:21:27</t>
         </is>
       </c>
       <c r="H13" s="1" t="inlineStr">
@@ -1264,7 +1264,7 @@
       </c>
       <c r="G14" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22 09:51:21</t>
+          <t>2026-05-26 00:21:27</t>
         </is>
       </c>
       <c r="H14" s="1" t="inlineStr">
@@ -1300,7 +1300,7 @@
       </c>
       <c r="G15" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22 09:51:21</t>
+          <t>2026-05-26 00:21:27</t>
         </is>
       </c>
       <c r="H15" s="1" t="inlineStr">
@@ -1336,7 +1336,7 @@
       </c>
       <c r="G16" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22 09:51:21</t>
+          <t>2026-05-26 00:21:27</t>
         </is>
       </c>
       <c r="H16" s="1" t="inlineStr">
@@ -1372,7 +1372,7 @@
       </c>
       <c r="G17" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22 09:51:21</t>
+          <t>2026-05-26 00:21:27</t>
         </is>
       </c>
       <c r="H17" s="1" t="inlineStr">
@@ -1408,7 +1408,7 @@
       </c>
       <c r="G18" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22 09:51:21</t>
+          <t>2026-05-26 00:21:27</t>
         </is>
       </c>
       <c r="H18" s="1" t="inlineStr">
@@ -1444,7 +1444,7 @@
       </c>
       <c r="G19" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22 09:51:21</t>
+          <t>2026-05-26 00:21:27</t>
         </is>
       </c>
       <c r="H19" s="1" t="inlineStr">
@@ -1480,7 +1480,7 @@
       </c>
       <c r="G20" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22 09:51:21</t>
+          <t>2026-05-26 00:21:27</t>
         </is>
       </c>
       <c r="H20" s="1" t="inlineStr">
@@ -1516,7 +1516,7 @@
       </c>
       <c r="G21" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22 09:51:21</t>
+          <t>2026-05-26 00:21:27</t>
         </is>
       </c>
       <c r="H21" s="1" t="inlineStr">
@@ -1552,7 +1552,7 @@
       </c>
       <c r="G22" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22 09:51:21</t>
+          <t>2026-05-26 00:21:27</t>
         </is>
       </c>
       <c r="H22" s="1" t="inlineStr">
@@ -1588,7 +1588,7 @@
       </c>
       <c r="G23" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22 09:51:21</t>
+          <t>2026-05-26 00:21:27</t>
         </is>
       </c>
       <c r="H23" s="1" t="inlineStr">
@@ -1624,7 +1624,7 @@
       </c>
       <c r="G24" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22 09:51:21</t>
+          <t>2026-05-26 00:21:27</t>
         </is>
       </c>
       <c r="H24" s="1" t="inlineStr">
@@ -1660,7 +1660,7 @@
       </c>
       <c r="G25" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22 09:51:21</t>
+          <t>2026-05-26 00:21:27</t>
         </is>
       </c>
       <c r="H25" s="1" t="inlineStr">
@@ -1696,7 +1696,7 @@
       </c>
       <c r="G26" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22 09:51:21</t>
+          <t>2026-05-26 00:21:27</t>
         </is>
       </c>
       <c r="H26" s="1" t="inlineStr">
@@ -1732,7 +1732,7 @@
       </c>
       <c r="G27" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22 09:51:21</t>
+          <t>2026-05-26 00:21:27</t>
         </is>
       </c>
       <c r="H27" s="1" t="inlineStr">
@@ -1768,7 +1768,7 @@
       </c>
       <c r="G28" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22 09:51:21</t>
+          <t>2026-05-26 00:21:27</t>
         </is>
       </c>
       <c r="H28" s="1" t="inlineStr">
@@ -1804,7 +1804,7 @@
       </c>
       <c r="G29" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22 09:51:21</t>
+          <t>2026-05-26 00:21:27</t>
         </is>
       </c>
       <c r="H29" s="1" t="inlineStr">
@@ -1840,7 +1840,7 @@
       </c>
       <c r="G30" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22 09:51:21</t>
+          <t>2026-05-26 00:21:27</t>
         </is>
       </c>
       <c r="H30" s="1" t="inlineStr">
@@ -1876,7 +1876,7 @@
       </c>
       <c r="G31" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22 09:51:21</t>
+          <t>2026-05-26 00:21:27</t>
         </is>
       </c>
       <c r="H31" s="1" t="inlineStr">
@@ -1912,7 +1912,7 @@
       </c>
       <c r="G32" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22 09:51:21</t>
+          <t>2026-05-26 00:21:27</t>
         </is>
       </c>
       <c r="H32" s="1" t="inlineStr">
@@ -1948,7 +1948,7 @@
       </c>
       <c r="G33" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22 09:51:21</t>
+          <t>2026-05-26 00:21:27</t>
         </is>
       </c>
       <c r="H33" s="1" t="inlineStr">
@@ -1984,7 +1984,7 @@
       </c>
       <c r="G34" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22 09:51:21</t>
+          <t>2026-05-26 00:21:27</t>
         </is>
       </c>
       <c r="H34" s="1" t="inlineStr">
@@ -2020,7 +2020,7 @@
       </c>
       <c r="G35" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22 09:51:21</t>
+          <t>2026-05-26 00:21:27</t>
         </is>
       </c>
       <c r="H35" s="1" t="inlineStr">
@@ -2056,7 +2056,7 @@
       </c>
       <c r="G36" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22 09:51:21</t>
+          <t>2026-05-26 00:21:27</t>
         </is>
       </c>
       <c r="H36" s="1" t="inlineStr">
@@ -2092,7 +2092,7 @@
       </c>
       <c r="G37" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22 09:51:21</t>
+          <t>2026-05-26 00:21:27</t>
         </is>
       </c>
       <c r="H37" s="1" t="inlineStr">
@@ -2128,7 +2128,7 @@
       </c>
       <c r="G38" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22 09:51:21</t>
+          <t>2026-05-26 00:21:27</t>
         </is>
       </c>
       <c r="H38" s="1" t="inlineStr">
@@ -2164,7 +2164,7 @@
       </c>
       <c r="G39" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22 09:51:21</t>
+          <t>2026-05-26 00:21:27</t>
         </is>
       </c>
       <c r="H39" s="1" t="inlineStr">
@@ -2200,7 +2200,7 @@
       </c>
       <c r="G40" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22 09:51:21</t>
+          <t>2026-05-26 00:21:27</t>
         </is>
       </c>
       <c r="H40" s="1" t="inlineStr">
@@ -2236,7 +2236,7 @@
       </c>
       <c r="G41" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22 09:51:21</t>
+          <t>2026-05-26 00:21:27</t>
         </is>
       </c>
       <c r="H41" s="1" t="inlineStr">
@@ -2272,7 +2272,7 @@
       </c>
       <c r="G42" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22 09:51:21</t>
+          <t>2026-05-26 00:21:27</t>
         </is>
       </c>
       <c r="H42" s="1" t="inlineStr">
@@ -2308,7 +2308,7 @@
       </c>
       <c r="G43" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22 09:51:21</t>
+          <t>2026-05-26 00:21:27</t>
         </is>
       </c>
       <c r="H43" s="1" t="inlineStr">
@@ -2344,7 +2344,7 @@
       </c>
       <c r="G44" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22 09:51:21</t>
+          <t>2026-05-26 00:21:27</t>
         </is>
       </c>
       <c r="H44" s="1" t="inlineStr">
@@ -2380,7 +2380,7 @@
       </c>
       <c r="G45" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22 09:51:21</t>
+          <t>2026-05-26 00:21:27</t>
         </is>
       </c>
       <c r="H45" s="1" t="inlineStr">
@@ -2416,7 +2416,7 @@
       </c>
       <c r="G46" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22 09:51:21</t>
+          <t>2026-05-26 00:21:27</t>
         </is>
       </c>
       <c r="H46" s="1" t="inlineStr">
@@ -2452,7 +2452,7 @@
       </c>
       <c r="G47" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22 09:51:21</t>
+          <t>2026-05-26 00:21:27</t>
         </is>
       </c>
       <c r="H47" s="1" t="inlineStr">
@@ -2488,7 +2488,7 @@
       </c>
       <c r="G48" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22 09:51:21</t>
+          <t>2026-05-26 00:21:27</t>
         </is>
       </c>
       <c r="H48" s="1" t="inlineStr">
@@ -2524,7 +2524,7 @@
       </c>
       <c r="G49" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22 09:51:21</t>
+          <t>2026-05-26 00:21:27</t>
         </is>
       </c>
       <c r="H49" s="1" t="inlineStr">
@@ -2560,7 +2560,7 @@
       </c>
       <c r="G50" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22 09:51:21</t>
+          <t>2026-05-26 00:21:27</t>
         </is>
       </c>
       <c r="H50" s="1" t="inlineStr">

</xml_diff>

<commit_message>
improve forecast speed and bot reliability
</commit_message>
<xml_diff>
--- a/ferniq_oportunidad_scraper/resultado_etapa_ferniq.xlsx
+++ b/ferniq_oportunidad_scraper/resultado_etapa_ferniq.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -597,7 +597,7 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>Jesus Cabello</t>
+          <t>Miguel Angel Haro</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
@@ -622,7 +622,7 @@
         <v>0</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>0</v>
+        <v>3499</v>
       </c>
       <c r="J5" s="2">
         <f>SUM(B5:I5)</f>
@@ -632,7 +632,7 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>Miguel Angel Haro</t>
+          <t>Paco Buendia</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -645,7 +645,7 @@
         <v>0</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>0</v>
+        <v>11999</v>
       </c>
       <c r="F6" s="2" t="n">
         <v>0</v>
@@ -657,7 +657,7 @@
         <v>0</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>3499</v>
+        <v>0</v>
       </c>
       <c r="J6" s="2">
         <f>SUM(B6:I6)</f>
@@ -667,7 +667,7 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>Paco Buendia</t>
+          <t>Ramon Jimenez</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
@@ -680,7 +680,7 @@
         <v>0</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>11999</v>
+        <v>1</v>
       </c>
       <c r="F7" s="2" t="n">
         <v>0</v>
@@ -700,52 +700,17 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>Ramon Jimenez</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="C8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="F8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="A8" s="1" t="n"/>
+      <c r="B8" s="1" t="n"/>
+      <c r="C8" s="1" t="n"/>
+      <c r="D8" s="1" t="n"/>
+      <c r="E8" s="1" t="n"/>
+      <c r="F8" s="1" t="n"/>
+      <c r="G8" s="1" t="n"/>
+      <c r="H8" s="1" t="n"/>
+      <c r="I8" s="1" t="n"/>
       <c r="J8" s="2">
-        <f>SUM(B8:I8)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="1" t="n"/>
-      <c r="B9" s="1" t="n"/>
-      <c r="C9" s="1" t="n"/>
-      <c r="D9" s="1" t="n"/>
-      <c r="E9" s="1" t="n"/>
-      <c r="F9" s="1" t="n"/>
-      <c r="G9" s="1" t="n"/>
-      <c r="H9" s="1" t="n"/>
-      <c r="I9" s="1" t="n"/>
-      <c r="J9" s="2">
-        <f>SUM(J2:J8)</f>
+        <f>SUM(J2:J7)</f>
         <v/>
       </c>
     </row>
@@ -760,7 +725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H50"/>
+  <dimension ref="A1:H49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -808,7 +773,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Agustin Parejo</t>
+          <t>Javier Barcelo</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -824,15 +789,15 @@
       <c r="D2" s="1" t="inlineStr"/>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>€0.00</t>
+          <t>€3,000.00</t>
         </is>
       </c>
       <c r="F2" s="1" t="n">
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="G2" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 00:21:27</t>
+          <t>2026-05-26 01:35:58</t>
         </is>
       </c>
       <c r="H2" s="1" t="inlineStr">
@@ -844,7 +809,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Agustin Parejo</t>
+          <t>Javier Barcelo</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -868,7 +833,7 @@
       </c>
       <c r="G3" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 00:21:27</t>
+          <t>2026-05-26 01:35:58</t>
         </is>
       </c>
       <c r="H3" s="1" t="inlineStr">
@@ -880,7 +845,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>Agustin Parejo</t>
+          <t>Javier Barcelo</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
@@ -904,7 +869,7 @@
       </c>
       <c r="G4" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 00:21:27</t>
+          <t>2026-05-26 01:35:58</t>
         </is>
       </c>
       <c r="H4" s="1" t="inlineStr">
@@ -916,7 +881,7 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>Agustin Parejo</t>
+          <t>Javier Barcelo</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
@@ -940,7 +905,7 @@
       </c>
       <c r="G5" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 00:21:27</t>
+          <t>2026-05-26 01:35:58</t>
         </is>
       </c>
       <c r="H5" s="1" t="inlineStr">
@@ -952,7 +917,7 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>Agustin Parejo</t>
+          <t>Javier Barcelo</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
@@ -976,7 +941,7 @@
       </c>
       <c r="G6" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 00:21:27</t>
+          <t>2026-05-26 01:35:58</t>
         </is>
       </c>
       <c r="H6" s="1" t="inlineStr">
@@ -988,7 +953,7 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>Agustin Parejo</t>
+          <t>Javier Barcelo</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr">
@@ -1012,7 +977,7 @@
       </c>
       <c r="G7" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 00:21:27</t>
+          <t>2026-05-26 01:35:58</t>
         </is>
       </c>
       <c r="H7" s="1" t="inlineStr">
@@ -1024,7 +989,7 @@
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>Agustin Parejo</t>
+          <t>Javier Barcelo</t>
         </is>
       </c>
       <c r="B8" s="1" t="inlineStr">
@@ -1048,7 +1013,7 @@
       </c>
       <c r="G8" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 00:21:27</t>
+          <t>2026-05-26 01:35:58</t>
         </is>
       </c>
       <c r="H8" s="1" t="inlineStr">
@@ -1060,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>Agustin Parejo</t>
+          <t>Javier Barcelo</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
@@ -1076,15 +1041,15 @@
       <c r="D9" s="1" t="inlineStr"/>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>€20,575.00</t>
+          <t>€9,000.00</t>
         </is>
       </c>
       <c r="F9" s="1" t="n">
-        <v>20575</v>
+        <v>9000</v>
       </c>
       <c r="G9" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 00:21:27</t>
+          <t>2026-05-26 01:35:58</t>
         </is>
       </c>
       <c r="H9" s="1" t="inlineStr">
@@ -1120,7 +1085,7 @@
       </c>
       <c r="G10" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 00:21:27</t>
+          <t>2026-05-26 01:35:58</t>
         </is>
       </c>
       <c r="H10" s="1" t="inlineStr">
@@ -1156,7 +1121,7 @@
       </c>
       <c r="G11" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 00:21:27</t>
+          <t>2026-05-26 01:35:58</t>
         </is>
       </c>
       <c r="H11" s="1" t="inlineStr">
@@ -1192,7 +1157,7 @@
       </c>
       <c r="G12" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 00:21:27</t>
+          <t>2026-05-26 01:35:58</t>
         </is>
       </c>
       <c r="H12" s="1" t="inlineStr">
@@ -1228,7 +1193,7 @@
       </c>
       <c r="G13" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 00:21:27</t>
+          <t>2026-05-26 01:35:58</t>
         </is>
       </c>
       <c r="H13" s="1" t="inlineStr">
@@ -1264,7 +1229,7 @@
       </c>
       <c r="G14" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 00:21:27</t>
+          <t>2026-05-26 01:35:58</t>
         </is>
       </c>
       <c r="H14" s="1" t="inlineStr">
@@ -1300,7 +1265,7 @@
       </c>
       <c r="G15" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 00:21:27</t>
+          <t>2026-05-26 01:35:58</t>
         </is>
       </c>
       <c r="H15" s="1" t="inlineStr">
@@ -1336,7 +1301,7 @@
       </c>
       <c r="G16" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 00:21:27</t>
+          <t>2026-05-26 01:35:58</t>
         </is>
       </c>
       <c r="H16" s="1" t="inlineStr">
@@ -1372,7 +1337,7 @@
       </c>
       <c r="G17" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 00:21:27</t>
+          <t>2026-05-26 01:35:58</t>
         </is>
       </c>
       <c r="H17" s="1" t="inlineStr">
@@ -1384,7 +1349,7 @@
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>Javier Barcelo</t>
+          <t>Agustin Parejo</t>
         </is>
       </c>
       <c r="B18" s="1" t="inlineStr">
@@ -1400,15 +1365,15 @@
       <c r="D18" s="1" t="inlineStr"/>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>€3,000.00</t>
+          <t>€0.00</t>
         </is>
       </c>
       <c r="F18" s="1" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="G18" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 00:21:27</t>
+          <t>2026-05-26 01:35:58</t>
         </is>
       </c>
       <c r="H18" s="1" t="inlineStr">
@@ -1420,7 +1385,7 @@
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>Javier Barcelo</t>
+          <t>Agustin Parejo</t>
         </is>
       </c>
       <c r="B19" s="1" t="inlineStr">
@@ -1444,7 +1409,7 @@
       </c>
       <c r="G19" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 00:21:27</t>
+          <t>2026-05-26 01:35:58</t>
         </is>
       </c>
       <c r="H19" s="1" t="inlineStr">
@@ -1456,7 +1421,7 @@
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>Javier Barcelo</t>
+          <t>Agustin Parejo</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr">
@@ -1480,7 +1445,7 @@
       </c>
       <c r="G20" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 00:21:27</t>
+          <t>2026-05-26 01:35:58</t>
         </is>
       </c>
       <c r="H20" s="1" t="inlineStr">
@@ -1492,7 +1457,7 @@
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>Javier Barcelo</t>
+          <t>Agustin Parejo</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr">
@@ -1516,7 +1481,7 @@
       </c>
       <c r="G21" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 00:21:27</t>
+          <t>2026-05-26 01:35:58</t>
         </is>
       </c>
       <c r="H21" s="1" t="inlineStr">
@@ -1528,7 +1493,7 @@
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>Javier Barcelo</t>
+          <t>Agustin Parejo</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
@@ -1552,7 +1517,7 @@
       </c>
       <c r="G22" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 00:21:27</t>
+          <t>2026-05-26 01:35:58</t>
         </is>
       </c>
       <c r="H22" s="1" t="inlineStr">
@@ -1564,7 +1529,7 @@
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>Javier Barcelo</t>
+          <t>Agustin Parejo</t>
         </is>
       </c>
       <c r="B23" s="1" t="inlineStr">
@@ -1588,7 +1553,7 @@
       </c>
       <c r="G23" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 00:21:27</t>
+          <t>2026-05-26 01:35:58</t>
         </is>
       </c>
       <c r="H23" s="1" t="inlineStr">
@@ -1600,7 +1565,7 @@
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>Javier Barcelo</t>
+          <t>Agustin Parejo</t>
         </is>
       </c>
       <c r="B24" s="1" t="inlineStr">
@@ -1624,7 +1589,7 @@
       </c>
       <c r="G24" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 00:21:27</t>
+          <t>2026-05-26 01:35:58</t>
         </is>
       </c>
       <c r="H24" s="1" t="inlineStr">
@@ -1636,7 +1601,7 @@
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>Javier Barcelo</t>
+          <t>Agustin Parejo</t>
         </is>
       </c>
       <c r="B25" s="1" t="inlineStr">
@@ -1652,15 +1617,15 @@
       <c r="D25" s="1" t="inlineStr"/>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>€9,000.00</t>
+          <t>€20,575.00</t>
         </is>
       </c>
       <c r="F25" s="1" t="n">
-        <v>9000</v>
+        <v>20575</v>
       </c>
       <c r="G25" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 00:21:27</t>
+          <t>2026-05-26 01:35:58</t>
         </is>
       </c>
       <c r="H25" s="1" t="inlineStr">
@@ -1672,7 +1637,7 @@
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>Jesus Cabello</t>
+          <t>Miguel Angel Haro</t>
         </is>
       </c>
       <c r="B26" s="1" t="inlineStr">
@@ -1682,7 +1647,7 @@
       </c>
       <c r="C26" s="1" t="inlineStr">
         <is>
-          <t>Proceso de compras</t>
+          <t>Aceptado</t>
         </is>
       </c>
       <c r="D26" s="1" t="inlineStr"/>
@@ -1696,12 +1661,12 @@
       </c>
       <c r="G26" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 00:21:27</t>
+          <t>2026-05-26 01:35:58</t>
         </is>
       </c>
       <c r="H26" s="1" t="inlineStr">
         <is>
-          <t>dom</t>
+          <t>dom_chart_click</t>
         </is>
       </c>
     </row>
@@ -1718,7 +1683,7 @@
       </c>
       <c r="C27" s="1" t="inlineStr">
         <is>
-          <t>Aceptado</t>
+          <t>Anulado / Perdido</t>
         </is>
       </c>
       <c r="D27" s="1" t="inlineStr"/>
@@ -1732,7 +1697,7 @@
       </c>
       <c r="G27" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 00:21:27</t>
+          <t>2026-05-26 01:35:58</t>
         </is>
       </c>
       <c r="H27" s="1" t="inlineStr">
@@ -1754,7 +1719,7 @@
       </c>
       <c r="C28" s="1" t="inlineStr">
         <is>
-          <t>Anulado / Perdido</t>
+          <t>Contacto inicial</t>
         </is>
       </c>
       <c r="D28" s="1" t="inlineStr"/>
@@ -1768,7 +1733,7 @@
       </c>
       <c r="G28" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 00:21:27</t>
+          <t>2026-05-26 01:35:58</t>
         </is>
       </c>
       <c r="H28" s="1" t="inlineStr">
@@ -1790,7 +1755,7 @@
       </c>
       <c r="C29" s="1" t="inlineStr">
         <is>
-          <t>Contacto inicial</t>
+          <t>Envio de presupuesto</t>
         </is>
       </c>
       <c r="D29" s="1" t="inlineStr"/>
@@ -1804,7 +1769,7 @@
       </c>
       <c r="G29" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 00:21:27</t>
+          <t>2026-05-26 01:35:58</t>
         </is>
       </c>
       <c r="H29" s="1" t="inlineStr">
@@ -1826,7 +1791,7 @@
       </c>
       <c r="C30" s="1" t="inlineStr">
         <is>
-          <t>Envio de presupuesto</t>
+          <t>Negociacion</t>
         </is>
       </c>
       <c r="D30" s="1" t="inlineStr"/>
@@ -1840,7 +1805,7 @@
       </c>
       <c r="G30" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 00:21:27</t>
+          <t>2026-05-26 01:35:58</t>
         </is>
       </c>
       <c r="H30" s="1" t="inlineStr">
@@ -1862,7 +1827,7 @@
       </c>
       <c r="C31" s="1" t="inlineStr">
         <is>
-          <t>Negociacion</t>
+          <t>Oportunidad de valor</t>
         </is>
       </c>
       <c r="D31" s="1" t="inlineStr"/>
@@ -1876,7 +1841,7 @@
       </c>
       <c r="G31" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 00:21:27</t>
+          <t>2026-05-26 01:35:58</t>
         </is>
       </c>
       <c r="H31" s="1" t="inlineStr">
@@ -1898,7 +1863,7 @@
       </c>
       <c r="C32" s="1" t="inlineStr">
         <is>
-          <t>Oportunidad de valor</t>
+          <t>Por confirmar / Sin respuesta</t>
         </is>
       </c>
       <c r="D32" s="1" t="inlineStr"/>
@@ -1912,7 +1877,7 @@
       </c>
       <c r="G32" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 00:21:27</t>
+          <t>2026-05-26 01:35:58</t>
         </is>
       </c>
       <c r="H32" s="1" t="inlineStr">
@@ -1934,21 +1899,21 @@
       </c>
       <c r="C33" s="1" t="inlineStr">
         <is>
-          <t>Por confirmar / Sin respuesta</t>
+          <t>Proceso de compras</t>
         </is>
       </c>
       <c r="D33" s="1" t="inlineStr"/>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>€0.00</t>
+          <t>€3,499.00</t>
         </is>
       </c>
       <c r="F33" s="1" t="n">
-        <v>0</v>
+        <v>3499</v>
       </c>
       <c r="G33" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 00:21:27</t>
+          <t>2026-05-26 01:35:58</t>
         </is>
       </c>
       <c r="H33" s="1" t="inlineStr">
@@ -1960,7 +1925,7 @@
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>Miguel Angel Haro</t>
+          <t>Paco Buendia</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
@@ -1970,21 +1935,21 @@
       </c>
       <c r="C34" s="1" t="inlineStr">
         <is>
-          <t>Proceso de compras</t>
+          <t>Aceptado</t>
         </is>
       </c>
       <c r="D34" s="1" t="inlineStr"/>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>€3,499.00</t>
+          <t>€0.00</t>
         </is>
       </c>
       <c r="F34" s="1" t="n">
-        <v>3499</v>
+        <v>0</v>
       </c>
       <c r="G34" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 00:21:27</t>
+          <t>2026-05-26 01:35:58</t>
         </is>
       </c>
       <c r="H34" s="1" t="inlineStr">
@@ -2006,7 +1971,7 @@
       </c>
       <c r="C35" s="1" t="inlineStr">
         <is>
-          <t>Aceptado</t>
+          <t>Anulado / Perdido</t>
         </is>
       </c>
       <c r="D35" s="1" t="inlineStr"/>
@@ -2020,7 +1985,7 @@
       </c>
       <c r="G35" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 00:21:27</t>
+          <t>2026-05-26 01:35:58</t>
         </is>
       </c>
       <c r="H35" s="1" t="inlineStr">
@@ -2042,7 +2007,7 @@
       </c>
       <c r="C36" s="1" t="inlineStr">
         <is>
-          <t>Anulado / Perdido</t>
+          <t>Contacto inicial</t>
         </is>
       </c>
       <c r="D36" s="1" t="inlineStr"/>
@@ -2056,7 +2021,7 @@
       </c>
       <c r="G36" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 00:21:27</t>
+          <t>2026-05-26 01:35:58</t>
         </is>
       </c>
       <c r="H36" s="1" t="inlineStr">
@@ -2078,21 +2043,21 @@
       </c>
       <c r="C37" s="1" t="inlineStr">
         <is>
-          <t>Contacto inicial</t>
+          <t>Envio de presupuesto</t>
         </is>
       </c>
       <c r="D37" s="1" t="inlineStr"/>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>€0.00</t>
+          <t>€11,999.00</t>
         </is>
       </c>
       <c r="F37" s="1" t="n">
-        <v>0</v>
+        <v>11999</v>
       </c>
       <c r="G37" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 00:21:27</t>
+          <t>2026-05-26 01:35:58</t>
         </is>
       </c>
       <c r="H37" s="1" t="inlineStr">
@@ -2114,21 +2079,21 @@
       </c>
       <c r="C38" s="1" t="inlineStr">
         <is>
-          <t>Envio de presupuesto</t>
+          <t>Negociacion</t>
         </is>
       </c>
       <c r="D38" s="1" t="inlineStr"/>
       <c r="E38" s="1" t="inlineStr">
         <is>
-          <t>€11,999.00</t>
+          <t>€0.00</t>
         </is>
       </c>
       <c r="F38" s="1" t="n">
-        <v>11999</v>
+        <v>0</v>
       </c>
       <c r="G38" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 00:21:27</t>
+          <t>2026-05-26 01:35:58</t>
         </is>
       </c>
       <c r="H38" s="1" t="inlineStr">
@@ -2150,7 +2115,7 @@
       </c>
       <c r="C39" s="1" t="inlineStr">
         <is>
-          <t>Negociacion</t>
+          <t>Oportunidad de valor</t>
         </is>
       </c>
       <c r="D39" s="1" t="inlineStr"/>
@@ -2164,7 +2129,7 @@
       </c>
       <c r="G39" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 00:21:27</t>
+          <t>2026-05-26 01:35:58</t>
         </is>
       </c>
       <c r="H39" s="1" t="inlineStr">
@@ -2186,7 +2151,7 @@
       </c>
       <c r="C40" s="1" t="inlineStr">
         <is>
-          <t>Oportunidad de valor</t>
+          <t>Por confirmar / Sin respuesta</t>
         </is>
       </c>
       <c r="D40" s="1" t="inlineStr"/>
@@ -2200,7 +2165,7 @@
       </c>
       <c r="G40" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 00:21:27</t>
+          <t>2026-05-26 01:35:58</t>
         </is>
       </c>
       <c r="H40" s="1" t="inlineStr">
@@ -2222,7 +2187,7 @@
       </c>
       <c r="C41" s="1" t="inlineStr">
         <is>
-          <t>Por confirmar / Sin respuesta</t>
+          <t>Proceso de compras</t>
         </is>
       </c>
       <c r="D41" s="1" t="inlineStr"/>
@@ -2236,7 +2201,7 @@
       </c>
       <c r="G41" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 00:21:27</t>
+          <t>2026-05-26 01:35:58</t>
         </is>
       </c>
       <c r="H41" s="1" t="inlineStr">
@@ -2248,7 +2213,7 @@
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>Paco Buendia</t>
+          <t>Ramon Jimenez</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">
@@ -2258,7 +2223,7 @@
       </c>
       <c r="C42" s="1" t="inlineStr">
         <is>
-          <t>Proceso de compras</t>
+          <t>Aceptado</t>
         </is>
       </c>
       <c r="D42" s="1" t="inlineStr"/>
@@ -2272,7 +2237,7 @@
       </c>
       <c r="G42" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 00:21:27</t>
+          <t>2026-05-26 01:35:58</t>
         </is>
       </c>
       <c r="H42" s="1" t="inlineStr">
@@ -2294,7 +2259,7 @@
       </c>
       <c r="C43" s="1" t="inlineStr">
         <is>
-          <t>Aceptado</t>
+          <t>Anulado / Perdido</t>
         </is>
       </c>
       <c r="D43" s="1" t="inlineStr"/>
@@ -2308,7 +2273,7 @@
       </c>
       <c r="G43" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 00:21:27</t>
+          <t>2026-05-26 01:35:58</t>
         </is>
       </c>
       <c r="H43" s="1" t="inlineStr">
@@ -2330,7 +2295,7 @@
       </c>
       <c r="C44" s="1" t="inlineStr">
         <is>
-          <t>Anulado / Perdido</t>
+          <t>Contacto inicial</t>
         </is>
       </c>
       <c r="D44" s="1" t="inlineStr"/>
@@ -2344,7 +2309,7 @@
       </c>
       <c r="G44" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 00:21:27</t>
+          <t>2026-05-26 01:35:58</t>
         </is>
       </c>
       <c r="H44" s="1" t="inlineStr">
@@ -2366,21 +2331,21 @@
       </c>
       <c r="C45" s="1" t="inlineStr">
         <is>
-          <t>Contacto inicial</t>
+          <t>Envio de presupuesto</t>
         </is>
       </c>
       <c r="D45" s="1" t="inlineStr"/>
       <c r="E45" s="1" t="inlineStr">
         <is>
-          <t>€0.00</t>
+          <t>€1.00</t>
         </is>
       </c>
       <c r="F45" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G45" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 00:21:27</t>
+          <t>2026-05-26 01:35:58</t>
         </is>
       </c>
       <c r="H45" s="1" t="inlineStr">
@@ -2402,21 +2367,21 @@
       </c>
       <c r="C46" s="1" t="inlineStr">
         <is>
-          <t>Envio de presupuesto</t>
+          <t>Negociacion</t>
         </is>
       </c>
       <c r="D46" s="1" t="inlineStr"/>
       <c r="E46" s="1" t="inlineStr">
         <is>
-          <t>€1.00</t>
+          <t>€0.00</t>
         </is>
       </c>
       <c r="F46" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G46" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 00:21:27</t>
+          <t>2026-05-26 01:35:58</t>
         </is>
       </c>
       <c r="H46" s="1" t="inlineStr">
@@ -2438,7 +2403,7 @@
       </c>
       <c r="C47" s="1" t="inlineStr">
         <is>
-          <t>Negociacion</t>
+          <t>Oportunidad de valor</t>
         </is>
       </c>
       <c r="D47" s="1" t="inlineStr"/>
@@ -2452,7 +2417,7 @@
       </c>
       <c r="G47" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 00:21:27</t>
+          <t>2026-05-26 01:35:58</t>
         </is>
       </c>
       <c r="H47" s="1" t="inlineStr">
@@ -2474,7 +2439,7 @@
       </c>
       <c r="C48" s="1" t="inlineStr">
         <is>
-          <t>Oportunidad de valor</t>
+          <t>Por confirmar / Sin respuesta</t>
         </is>
       </c>
       <c r="D48" s="1" t="inlineStr"/>
@@ -2488,7 +2453,7 @@
       </c>
       <c r="G48" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 00:21:27</t>
+          <t>2026-05-26 01:35:58</t>
         </is>
       </c>
       <c r="H48" s="1" t="inlineStr">
@@ -2510,7 +2475,7 @@
       </c>
       <c r="C49" s="1" t="inlineStr">
         <is>
-          <t>Por confirmar / Sin respuesta</t>
+          <t>Proceso de compras</t>
         </is>
       </c>
       <c r="D49" s="1" t="inlineStr"/>
@@ -2524,46 +2489,10 @@
       </c>
       <c r="G49" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 00:21:27</t>
+          <t>2026-05-26 01:35:58</t>
         </is>
       </c>
       <c r="H49" s="1" t="inlineStr">
-        <is>
-          <t>dom_chart_click</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="1" t="inlineStr">
-        <is>
-          <t>Ramon Jimenez</t>
-        </is>
-      </c>
-      <c r="B50" s="1" t="inlineStr">
-        <is>
-          <t>Mayo 2026</t>
-        </is>
-      </c>
-      <c r="C50" s="1" t="inlineStr">
-        <is>
-          <t>Proceso de compras</t>
-        </is>
-      </c>
-      <c r="D50" s="1" t="inlineStr"/>
-      <c r="E50" s="1" t="inlineStr">
-        <is>
-          <t>€0.00</t>
-        </is>
-      </c>
-      <c r="F50" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G50" s="1" t="inlineStr">
-        <is>
-          <t>2026-05-26 00:21:27</t>
-        </is>
-      </c>
-      <c r="H50" s="1" t="inlineStr">
         <is>
           <t>dom_chart_click</t>
         </is>

</xml_diff>

<commit_message>
Update stage and forecast bot outputs
</commit_message>
<xml_diff>
--- a/ferniq_oportunidad_scraper/resultado_etapa_ferniq.xlsx
+++ b/ferniq_oportunidad_scraper/resultado_etapa_ferniq.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Resumen" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Detalle" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detalle" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,8 +17,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="#,##0 €"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="#.##0,00 €"/>
+    <numFmt numFmtId="165" formatCode="#.##0"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -49,12 +50,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -422,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -492,7 +496,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Agustin Parejo</t>
+          <t>Ismael Serrano</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -517,7 +521,7 @@
         <v>0</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>20575</v>
+        <v>7500</v>
       </c>
       <c r="J2" s="2">
         <f>SUM(B2:I2)</f>
@@ -527,11 +531,11 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Ismael Serrano</t>
+          <t>Javier Barcelo</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="C3" s="2" t="n">
         <v>0</v>
@@ -552,7 +556,7 @@
         <v>0</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>7500</v>
+        <v>9000</v>
       </c>
       <c r="J3" s="2">
         <f>SUM(B3:I3)</f>
@@ -562,11 +566,11 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>Javier Barcelo</t>
+          <t>Jesus Cabello</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="C4" s="2" t="n">
         <v>0</v>
@@ -587,7 +591,7 @@
         <v>0</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>9000</v>
+        <v>0</v>
       </c>
       <c r="J4" s="2">
         <f>SUM(B4:I4)</f>
@@ -667,7 +671,7 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>Ramon Jimenez</t>
+          <t>Agustin Parejo</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
@@ -680,7 +684,7 @@
         <v>0</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F7" s="2" t="n">
         <v>0</v>
@@ -692,7 +696,7 @@
         <v>0</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>0</v>
+        <v>20575</v>
       </c>
       <c r="J7" s="2">
         <f>SUM(B7:I7)</f>
@@ -700,17 +704,87 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n"/>
-      <c r="B8" s="1" t="n"/>
-      <c r="C8" s="1" t="n"/>
-      <c r="D8" s="1" t="n"/>
-      <c r="E8" s="1" t="n"/>
-      <c r="F8" s="1" t="n"/>
-      <c r="G8" s="1" t="n"/>
-      <c r="H8" s="1" t="n"/>
-      <c r="I8" s="1" t="n"/>
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>Ramon Jimenez</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="J8" s="2">
-        <f>SUM(J2:J7)</f>
+        <f>SUM(B8:I8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>Daniel Amparan</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="2">
+        <f>SUM(B9:I9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="n"/>
+      <c r="B10" s="1" t="n"/>
+      <c r="C10" s="1" t="n"/>
+      <c r="D10" s="1" t="n"/>
+      <c r="E10" s="1" t="n"/>
+      <c r="F10" s="1" t="n"/>
+      <c r="G10" s="1" t="n"/>
+      <c r="H10" s="1" t="n"/>
+      <c r="I10" s="1" t="n"/>
+      <c r="J10" s="2">
+        <f>SUM(J2:J9)</f>
         <v/>
       </c>
     </row>
@@ -773,7 +847,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Javier Barcelo</t>
+          <t>Ismael Serrano</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -786,18 +860,18 @@
           <t>Aceptado</t>
         </is>
       </c>
-      <c r="D2" s="1" t="inlineStr"/>
+      <c r="D2" s="3" t="inlineStr"/>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>€3,000.00</t>
-        </is>
-      </c>
-      <c r="F2" s="1" t="n">
-        <v>3000</v>
+          <t>€0.00</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="G2" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 01:35:58</t>
+          <t>2026-05-26 10:03:09</t>
         </is>
       </c>
       <c r="H2" s="1" t="inlineStr">
@@ -809,7 +883,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Javier Barcelo</t>
+          <t>Ismael Serrano</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -822,18 +896,18 @@
           <t>Anulado / Perdido</t>
         </is>
       </c>
-      <c r="D3" s="1" t="inlineStr"/>
+      <c r="D3" s="3" t="inlineStr"/>
       <c r="E3" s="1" t="inlineStr">
         <is>
           <t>€0.00</t>
         </is>
       </c>
-      <c r="F3" s="1" t="n">
+      <c r="F3" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G3" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 01:35:58</t>
+          <t>2026-05-26 10:03:09</t>
         </is>
       </c>
       <c r="H3" s="1" t="inlineStr">
@@ -845,7 +919,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>Javier Barcelo</t>
+          <t>Ismael Serrano</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
@@ -858,18 +932,18 @@
           <t>Contacto inicial</t>
         </is>
       </c>
-      <c r="D4" s="1" t="inlineStr"/>
+      <c r="D4" s="3" t="inlineStr"/>
       <c r="E4" s="1" t="inlineStr">
         <is>
           <t>€0.00</t>
         </is>
       </c>
-      <c r="F4" s="1" t="n">
+      <c r="F4" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G4" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 01:35:58</t>
+          <t>2026-05-26 10:03:09</t>
         </is>
       </c>
       <c r="H4" s="1" t="inlineStr">
@@ -881,7 +955,7 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>Javier Barcelo</t>
+          <t>Ismael Serrano</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
@@ -894,18 +968,18 @@
           <t>Envio de presupuesto</t>
         </is>
       </c>
-      <c r="D5" s="1" t="inlineStr"/>
+      <c r="D5" s="3" t="inlineStr"/>
       <c r="E5" s="1" t="inlineStr">
         <is>
           <t>€0.00</t>
         </is>
       </c>
-      <c r="F5" s="1" t="n">
+      <c r="F5" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G5" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 01:35:58</t>
+          <t>2026-05-26 10:03:09</t>
         </is>
       </c>
       <c r="H5" s="1" t="inlineStr">
@@ -917,7 +991,7 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>Javier Barcelo</t>
+          <t>Ismael Serrano</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
@@ -930,18 +1004,18 @@
           <t>Negociacion</t>
         </is>
       </c>
-      <c r="D6" s="1" t="inlineStr"/>
+      <c r="D6" s="3" t="inlineStr"/>
       <c r="E6" s="1" t="inlineStr">
         <is>
           <t>€0.00</t>
         </is>
       </c>
-      <c r="F6" s="1" t="n">
+      <c r="F6" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G6" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 01:35:58</t>
+          <t>2026-05-26 10:03:09</t>
         </is>
       </c>
       <c r="H6" s="1" t="inlineStr">
@@ -953,7 +1027,7 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>Javier Barcelo</t>
+          <t>Ismael Serrano</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr">
@@ -966,18 +1040,18 @@
           <t>Oportunidad de valor</t>
         </is>
       </c>
-      <c r="D7" s="1" t="inlineStr"/>
+      <c r="D7" s="3" t="inlineStr"/>
       <c r="E7" s="1" t="inlineStr">
         <is>
           <t>€0.00</t>
         </is>
       </c>
-      <c r="F7" s="1" t="n">
+      <c r="F7" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G7" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 01:35:58</t>
+          <t>2026-05-26 10:03:09</t>
         </is>
       </c>
       <c r="H7" s="1" t="inlineStr">
@@ -989,7 +1063,7 @@
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>Javier Barcelo</t>
+          <t>Ismael Serrano</t>
         </is>
       </c>
       <c r="B8" s="1" t="inlineStr">
@@ -1002,18 +1076,18 @@
           <t>Por confirmar / Sin respuesta</t>
         </is>
       </c>
-      <c r="D8" s="1" t="inlineStr"/>
+      <c r="D8" s="3" t="inlineStr"/>
       <c r="E8" s="1" t="inlineStr">
         <is>
           <t>€0.00</t>
         </is>
       </c>
-      <c r="F8" s="1" t="n">
+      <c r="F8" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G8" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 01:35:58</t>
+          <t>2026-05-26 10:03:09</t>
         </is>
       </c>
       <c r="H8" s="1" t="inlineStr">
@@ -1025,7 +1099,7 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>Javier Barcelo</t>
+          <t>Ismael Serrano</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
@@ -1038,18 +1112,18 @@
           <t>Proceso de compras</t>
         </is>
       </c>
-      <c r="D9" s="1" t="inlineStr"/>
+      <c r="D9" s="3" t="inlineStr"/>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>€9,000.00</t>
-        </is>
-      </c>
-      <c r="F9" s="1" t="n">
-        <v>9000</v>
+          <t>€7,500.00</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>7500</v>
       </c>
       <c r="G9" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 01:35:58</t>
+          <t>2026-05-26 10:03:09</t>
         </is>
       </c>
       <c r="H9" s="1" t="inlineStr">
@@ -1061,7 +1135,7 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>Ismael Serrano</t>
+          <t>Javier Barcelo</t>
         </is>
       </c>
       <c r="B10" s="1" t="inlineStr">
@@ -1074,18 +1148,18 @@
           <t>Aceptado</t>
         </is>
       </c>
-      <c r="D10" s="1" t="inlineStr"/>
+      <c r="D10" s="3" t="inlineStr"/>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>€0.00</t>
-        </is>
-      </c>
-      <c r="F10" s="1" t="n">
-        <v>0</v>
+          <t>€3,000.00</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>3000</v>
       </c>
       <c r="G10" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 01:35:58</t>
+          <t>2026-05-26 10:03:09</t>
         </is>
       </c>
       <c r="H10" s="1" t="inlineStr">
@@ -1097,7 +1171,7 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>Ismael Serrano</t>
+          <t>Javier Barcelo</t>
         </is>
       </c>
       <c r="B11" s="1" t="inlineStr">
@@ -1110,18 +1184,18 @@
           <t>Anulado / Perdido</t>
         </is>
       </c>
-      <c r="D11" s="1" t="inlineStr"/>
+      <c r="D11" s="3" t="inlineStr"/>
       <c r="E11" s="1" t="inlineStr">
         <is>
           <t>€0.00</t>
         </is>
       </c>
-      <c r="F11" s="1" t="n">
+      <c r="F11" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G11" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 01:35:58</t>
+          <t>2026-05-26 10:03:09</t>
         </is>
       </c>
       <c r="H11" s="1" t="inlineStr">
@@ -1133,7 +1207,7 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>Ismael Serrano</t>
+          <t>Javier Barcelo</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
@@ -1146,18 +1220,18 @@
           <t>Contacto inicial</t>
         </is>
       </c>
-      <c r="D12" s="1" t="inlineStr"/>
+      <c r="D12" s="3" t="inlineStr"/>
       <c r="E12" s="1" t="inlineStr">
         <is>
           <t>€0.00</t>
         </is>
       </c>
-      <c r="F12" s="1" t="n">
+      <c r="F12" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G12" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 01:35:58</t>
+          <t>2026-05-26 10:03:09</t>
         </is>
       </c>
       <c r="H12" s="1" t="inlineStr">
@@ -1169,7 +1243,7 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>Ismael Serrano</t>
+          <t>Javier Barcelo</t>
         </is>
       </c>
       <c r="B13" s="1" t="inlineStr">
@@ -1182,18 +1256,18 @@
           <t>Envio de presupuesto</t>
         </is>
       </c>
-      <c r="D13" s="1" t="inlineStr"/>
+      <c r="D13" s="3" t="inlineStr"/>
       <c r="E13" s="1" t="inlineStr">
         <is>
           <t>€0.00</t>
         </is>
       </c>
-      <c r="F13" s="1" t="n">
+      <c r="F13" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G13" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 01:35:58</t>
+          <t>2026-05-26 10:03:09</t>
         </is>
       </c>
       <c r="H13" s="1" t="inlineStr">
@@ -1205,7 +1279,7 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>Ismael Serrano</t>
+          <t>Javier Barcelo</t>
         </is>
       </c>
       <c r="B14" s="1" t="inlineStr">
@@ -1218,18 +1292,18 @@
           <t>Negociacion</t>
         </is>
       </c>
-      <c r="D14" s="1" t="inlineStr"/>
+      <c r="D14" s="3" t="inlineStr"/>
       <c r="E14" s="1" t="inlineStr">
         <is>
           <t>€0.00</t>
         </is>
       </c>
-      <c r="F14" s="1" t="n">
+      <c r="F14" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G14" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 01:35:58</t>
+          <t>2026-05-26 10:03:09</t>
         </is>
       </c>
       <c r="H14" s="1" t="inlineStr">
@@ -1241,7 +1315,7 @@
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>Ismael Serrano</t>
+          <t>Javier Barcelo</t>
         </is>
       </c>
       <c r="B15" s="1" t="inlineStr">
@@ -1254,18 +1328,18 @@
           <t>Oportunidad de valor</t>
         </is>
       </c>
-      <c r="D15" s="1" t="inlineStr"/>
+      <c r="D15" s="3" t="inlineStr"/>
       <c r="E15" s="1" t="inlineStr">
         <is>
           <t>€0.00</t>
         </is>
       </c>
-      <c r="F15" s="1" t="n">
+      <c r="F15" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G15" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 01:35:58</t>
+          <t>2026-05-26 10:03:09</t>
         </is>
       </c>
       <c r="H15" s="1" t="inlineStr">
@@ -1277,7 +1351,7 @@
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>Ismael Serrano</t>
+          <t>Javier Barcelo</t>
         </is>
       </c>
       <c r="B16" s="1" t="inlineStr">
@@ -1290,18 +1364,18 @@
           <t>Por confirmar / Sin respuesta</t>
         </is>
       </c>
-      <c r="D16" s="1" t="inlineStr"/>
+      <c r="D16" s="3" t="inlineStr"/>
       <c r="E16" s="1" t="inlineStr">
         <is>
           <t>€0.00</t>
         </is>
       </c>
-      <c r="F16" s="1" t="n">
+      <c r="F16" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G16" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 01:35:58</t>
+          <t>2026-05-26 10:03:09</t>
         </is>
       </c>
       <c r="H16" s="1" t="inlineStr">
@@ -1313,7 +1387,7 @@
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>Ismael Serrano</t>
+          <t>Javier Barcelo</t>
         </is>
       </c>
       <c r="B17" s="1" t="inlineStr">
@@ -1326,18 +1400,18 @@
           <t>Proceso de compras</t>
         </is>
       </c>
-      <c r="D17" s="1" t="inlineStr"/>
+      <c r="D17" s="3" t="inlineStr"/>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>€7,500.00</t>
-        </is>
-      </c>
-      <c r="F17" s="1" t="n">
-        <v>7500</v>
+          <t>€9,000.00</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="n">
+        <v>9000</v>
       </c>
       <c r="G17" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 01:35:58</t>
+          <t>2026-05-26 10:03:09</t>
         </is>
       </c>
       <c r="H17" s="1" t="inlineStr">
@@ -1362,18 +1436,18 @@
           <t>Aceptado</t>
         </is>
       </c>
-      <c r="D18" s="1" t="inlineStr"/>
+      <c r="D18" s="3" t="inlineStr"/>
       <c r="E18" s="1" t="inlineStr">
         <is>
           <t>€0.00</t>
         </is>
       </c>
-      <c r="F18" s="1" t="n">
+      <c r="F18" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G18" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 01:35:58</t>
+          <t>2026-05-26 10:03:09</t>
         </is>
       </c>
       <c r="H18" s="1" t="inlineStr">
@@ -1398,18 +1472,18 @@
           <t>Anulado / Perdido</t>
         </is>
       </c>
-      <c r="D19" s="1" t="inlineStr"/>
+      <c r="D19" s="3" t="inlineStr"/>
       <c r="E19" s="1" t="inlineStr">
         <is>
           <t>€0.00</t>
         </is>
       </c>
-      <c r="F19" s="1" t="n">
+      <c r="F19" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G19" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 01:35:58</t>
+          <t>2026-05-26 10:03:09</t>
         </is>
       </c>
       <c r="H19" s="1" t="inlineStr">
@@ -1434,18 +1508,18 @@
           <t>Contacto inicial</t>
         </is>
       </c>
-      <c r="D20" s="1" t="inlineStr"/>
+      <c r="D20" s="3" t="inlineStr"/>
       <c r="E20" s="1" t="inlineStr">
         <is>
           <t>€0.00</t>
         </is>
       </c>
-      <c r="F20" s="1" t="n">
+      <c r="F20" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G20" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 01:35:58</t>
+          <t>2026-05-26 10:03:09</t>
         </is>
       </c>
       <c r="H20" s="1" t="inlineStr">
@@ -1470,18 +1544,18 @@
           <t>Envio de presupuesto</t>
         </is>
       </c>
-      <c r="D21" s="1" t="inlineStr"/>
+      <c r="D21" s="3" t="inlineStr"/>
       <c r="E21" s="1" t="inlineStr">
         <is>
           <t>€0.00</t>
         </is>
       </c>
-      <c r="F21" s="1" t="n">
+      <c r="F21" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G21" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 01:35:58</t>
+          <t>2026-05-26 10:03:09</t>
         </is>
       </c>
       <c r="H21" s="1" t="inlineStr">
@@ -1506,18 +1580,18 @@
           <t>Negociacion</t>
         </is>
       </c>
-      <c r="D22" s="1" t="inlineStr"/>
+      <c r="D22" s="3" t="inlineStr"/>
       <c r="E22" s="1" t="inlineStr">
         <is>
           <t>€0.00</t>
         </is>
       </c>
-      <c r="F22" s="1" t="n">
+      <c r="F22" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G22" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 01:35:58</t>
+          <t>2026-05-26 10:03:09</t>
         </is>
       </c>
       <c r="H22" s="1" t="inlineStr">
@@ -1542,18 +1616,18 @@
           <t>Oportunidad de valor</t>
         </is>
       </c>
-      <c r="D23" s="1" t="inlineStr"/>
+      <c r="D23" s="3" t="inlineStr"/>
       <c r="E23" s="1" t="inlineStr">
         <is>
           <t>€0.00</t>
         </is>
       </c>
-      <c r="F23" s="1" t="n">
+      <c r="F23" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G23" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 01:35:58</t>
+          <t>2026-05-26 10:03:09</t>
         </is>
       </c>
       <c r="H23" s="1" t="inlineStr">
@@ -1578,18 +1652,18 @@
           <t>Por confirmar / Sin respuesta</t>
         </is>
       </c>
-      <c r="D24" s="1" t="inlineStr"/>
+      <c r="D24" s="3" t="inlineStr"/>
       <c r="E24" s="1" t="inlineStr">
         <is>
           <t>€0.00</t>
         </is>
       </c>
-      <c r="F24" s="1" t="n">
+      <c r="F24" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G24" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 01:35:58</t>
+          <t>2026-05-26 10:03:09</t>
         </is>
       </c>
       <c r="H24" s="1" t="inlineStr">
@@ -1614,18 +1688,18 @@
           <t>Proceso de compras</t>
         </is>
       </c>
-      <c r="D25" s="1" t="inlineStr"/>
+      <c r="D25" s="3" t="inlineStr"/>
       <c r="E25" s="1" t="inlineStr">
         <is>
           <t>€20,575.00</t>
         </is>
       </c>
-      <c r="F25" s="1" t="n">
+      <c r="F25" s="2" t="n">
         <v>20575</v>
       </c>
       <c r="G25" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 01:35:58</t>
+          <t>2026-05-26 10:03:09</t>
         </is>
       </c>
       <c r="H25" s="1" t="inlineStr">
@@ -1650,18 +1724,18 @@
           <t>Aceptado</t>
         </is>
       </c>
-      <c r="D26" s="1" t="inlineStr"/>
+      <c r="D26" s="3" t="inlineStr"/>
       <c r="E26" s="1" t="inlineStr">
         <is>
           <t>€0.00</t>
         </is>
       </c>
-      <c r="F26" s="1" t="n">
+      <c r="F26" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G26" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 01:35:58</t>
+          <t>2026-05-26 10:03:09</t>
         </is>
       </c>
       <c r="H26" s="1" t="inlineStr">
@@ -1686,18 +1760,18 @@
           <t>Anulado / Perdido</t>
         </is>
       </c>
-      <c r="D27" s="1" t="inlineStr"/>
+      <c r="D27" s="3" t="inlineStr"/>
       <c r="E27" s="1" t="inlineStr">
         <is>
           <t>€0.00</t>
         </is>
       </c>
-      <c r="F27" s="1" t="n">
+      <c r="F27" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G27" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 01:35:58</t>
+          <t>2026-05-26 10:03:09</t>
         </is>
       </c>
       <c r="H27" s="1" t="inlineStr">
@@ -1722,18 +1796,18 @@
           <t>Contacto inicial</t>
         </is>
       </c>
-      <c r="D28" s="1" t="inlineStr"/>
+      <c r="D28" s="3" t="inlineStr"/>
       <c r="E28" s="1" t="inlineStr">
         <is>
           <t>€0.00</t>
         </is>
       </c>
-      <c r="F28" s="1" t="n">
+      <c r="F28" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G28" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 01:35:58</t>
+          <t>2026-05-26 10:03:09</t>
         </is>
       </c>
       <c r="H28" s="1" t="inlineStr">
@@ -1758,18 +1832,18 @@
           <t>Envio de presupuesto</t>
         </is>
       </c>
-      <c r="D29" s="1" t="inlineStr"/>
+      <c r="D29" s="3" t="inlineStr"/>
       <c r="E29" s="1" t="inlineStr">
         <is>
           <t>€0.00</t>
         </is>
       </c>
-      <c r="F29" s="1" t="n">
+      <c r="F29" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G29" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 01:35:58</t>
+          <t>2026-05-26 10:03:09</t>
         </is>
       </c>
       <c r="H29" s="1" t="inlineStr">
@@ -1794,18 +1868,18 @@
           <t>Negociacion</t>
         </is>
       </c>
-      <c r="D30" s="1" t="inlineStr"/>
+      <c r="D30" s="3" t="inlineStr"/>
       <c r="E30" s="1" t="inlineStr">
         <is>
           <t>€0.00</t>
         </is>
       </c>
-      <c r="F30" s="1" t="n">
+      <c r="F30" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G30" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 01:35:58</t>
+          <t>2026-05-26 10:03:09</t>
         </is>
       </c>
       <c r="H30" s="1" t="inlineStr">
@@ -1830,18 +1904,18 @@
           <t>Oportunidad de valor</t>
         </is>
       </c>
-      <c r="D31" s="1" t="inlineStr"/>
+      <c r="D31" s="3" t="inlineStr"/>
       <c r="E31" s="1" t="inlineStr">
         <is>
           <t>€0.00</t>
         </is>
       </c>
-      <c r="F31" s="1" t="n">
+      <c r="F31" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G31" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 01:35:58</t>
+          <t>2026-05-26 10:03:09</t>
         </is>
       </c>
       <c r="H31" s="1" t="inlineStr">
@@ -1866,18 +1940,18 @@
           <t>Por confirmar / Sin respuesta</t>
         </is>
       </c>
-      <c r="D32" s="1" t="inlineStr"/>
+      <c r="D32" s="3" t="inlineStr"/>
       <c r="E32" s="1" t="inlineStr">
         <is>
           <t>€0.00</t>
         </is>
       </c>
-      <c r="F32" s="1" t="n">
+      <c r="F32" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G32" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 01:35:58</t>
+          <t>2026-05-26 10:03:09</t>
         </is>
       </c>
       <c r="H32" s="1" t="inlineStr">
@@ -1902,18 +1976,18 @@
           <t>Proceso de compras</t>
         </is>
       </c>
-      <c r="D33" s="1" t="inlineStr"/>
+      <c r="D33" s="3" t="inlineStr"/>
       <c r="E33" s="1" t="inlineStr">
         <is>
           <t>€3,499.00</t>
         </is>
       </c>
-      <c r="F33" s="1" t="n">
+      <c r="F33" s="2" t="n">
         <v>3499</v>
       </c>
       <c r="G33" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 01:35:58</t>
+          <t>2026-05-26 10:03:09</t>
         </is>
       </c>
       <c r="H33" s="1" t="inlineStr">
@@ -1938,18 +2012,18 @@
           <t>Aceptado</t>
         </is>
       </c>
-      <c r="D34" s="1" t="inlineStr"/>
+      <c r="D34" s="3" t="inlineStr"/>
       <c r="E34" s="1" t="inlineStr">
         <is>
           <t>€0.00</t>
         </is>
       </c>
-      <c r="F34" s="1" t="n">
+      <c r="F34" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G34" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 01:35:58</t>
+          <t>2026-05-26 10:03:09</t>
         </is>
       </c>
       <c r="H34" s="1" t="inlineStr">
@@ -1974,18 +2048,18 @@
           <t>Anulado / Perdido</t>
         </is>
       </c>
-      <c r="D35" s="1" t="inlineStr"/>
+      <c r="D35" s="3" t="inlineStr"/>
       <c r="E35" s="1" t="inlineStr">
         <is>
           <t>€0.00</t>
         </is>
       </c>
-      <c r="F35" s="1" t="n">
+      <c r="F35" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G35" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 01:35:58</t>
+          <t>2026-05-26 10:03:09</t>
         </is>
       </c>
       <c r="H35" s="1" t="inlineStr">
@@ -2010,18 +2084,18 @@
           <t>Contacto inicial</t>
         </is>
       </c>
-      <c r="D36" s="1" t="inlineStr"/>
+      <c r="D36" s="3" t="inlineStr"/>
       <c r="E36" s="1" t="inlineStr">
         <is>
           <t>€0.00</t>
         </is>
       </c>
-      <c r="F36" s="1" t="n">
+      <c r="F36" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G36" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 01:35:58</t>
+          <t>2026-05-26 10:03:09</t>
         </is>
       </c>
       <c r="H36" s="1" t="inlineStr">
@@ -2046,18 +2120,18 @@
           <t>Envio de presupuesto</t>
         </is>
       </c>
-      <c r="D37" s="1" t="inlineStr"/>
+      <c r="D37" s="3" t="inlineStr"/>
       <c r="E37" s="1" t="inlineStr">
         <is>
           <t>€11,999.00</t>
         </is>
       </c>
-      <c r="F37" s="1" t="n">
+      <c r="F37" s="2" t="n">
         <v>11999</v>
       </c>
       <c r="G37" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 01:35:58</t>
+          <t>2026-05-26 10:03:09</t>
         </is>
       </c>
       <c r="H37" s="1" t="inlineStr">
@@ -2082,18 +2156,18 @@
           <t>Negociacion</t>
         </is>
       </c>
-      <c r="D38" s="1" t="inlineStr"/>
+      <c r="D38" s="3" t="inlineStr"/>
       <c r="E38" s="1" t="inlineStr">
         <is>
           <t>€0.00</t>
         </is>
       </c>
-      <c r="F38" s="1" t="n">
+      <c r="F38" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G38" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 01:35:58</t>
+          <t>2026-05-26 10:03:09</t>
         </is>
       </c>
       <c r="H38" s="1" t="inlineStr">
@@ -2118,18 +2192,18 @@
           <t>Oportunidad de valor</t>
         </is>
       </c>
-      <c r="D39" s="1" t="inlineStr"/>
+      <c r="D39" s="3" t="inlineStr"/>
       <c r="E39" s="1" t="inlineStr">
         <is>
           <t>€0.00</t>
         </is>
       </c>
-      <c r="F39" s="1" t="n">
+      <c r="F39" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G39" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 01:35:58</t>
+          <t>2026-05-26 10:03:09</t>
         </is>
       </c>
       <c r="H39" s="1" t="inlineStr">
@@ -2154,18 +2228,18 @@
           <t>Por confirmar / Sin respuesta</t>
         </is>
       </c>
-      <c r="D40" s="1" t="inlineStr"/>
+      <c r="D40" s="3" t="inlineStr"/>
       <c r="E40" s="1" t="inlineStr">
         <is>
           <t>€0.00</t>
         </is>
       </c>
-      <c r="F40" s="1" t="n">
+      <c r="F40" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G40" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 01:35:58</t>
+          <t>2026-05-26 10:03:09</t>
         </is>
       </c>
       <c r="H40" s="1" t="inlineStr">
@@ -2190,18 +2264,18 @@
           <t>Proceso de compras</t>
         </is>
       </c>
-      <c r="D41" s="1" t="inlineStr"/>
+      <c r="D41" s="3" t="inlineStr"/>
       <c r="E41" s="1" t="inlineStr">
         <is>
           <t>€0.00</t>
         </is>
       </c>
-      <c r="F41" s="1" t="n">
+      <c r="F41" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G41" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 01:35:58</t>
+          <t>2026-05-26 10:03:09</t>
         </is>
       </c>
       <c r="H41" s="1" t="inlineStr">
@@ -2226,18 +2300,18 @@
           <t>Aceptado</t>
         </is>
       </c>
-      <c r="D42" s="1" t="inlineStr"/>
+      <c r="D42" s="3" t="inlineStr"/>
       <c r="E42" s="1" t="inlineStr">
         <is>
           <t>€0.00</t>
         </is>
       </c>
-      <c r="F42" s="1" t="n">
+      <c r="F42" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G42" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 01:35:58</t>
+          <t>2026-05-26 10:03:09</t>
         </is>
       </c>
       <c r="H42" s="1" t="inlineStr">
@@ -2262,18 +2336,18 @@
           <t>Anulado / Perdido</t>
         </is>
       </c>
-      <c r="D43" s="1" t="inlineStr"/>
+      <c r="D43" s="3" t="inlineStr"/>
       <c r="E43" s="1" t="inlineStr">
         <is>
           <t>€0.00</t>
         </is>
       </c>
-      <c r="F43" s="1" t="n">
+      <c r="F43" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G43" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 01:35:58</t>
+          <t>2026-05-26 10:03:09</t>
         </is>
       </c>
       <c r="H43" s="1" t="inlineStr">
@@ -2298,18 +2372,18 @@
           <t>Contacto inicial</t>
         </is>
       </c>
-      <c r="D44" s="1" t="inlineStr"/>
+      <c r="D44" s="3" t="inlineStr"/>
       <c r="E44" s="1" t="inlineStr">
         <is>
           <t>€0.00</t>
         </is>
       </c>
-      <c r="F44" s="1" t="n">
+      <c r="F44" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G44" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 01:35:58</t>
+          <t>2026-05-26 10:03:09</t>
         </is>
       </c>
       <c r="H44" s="1" t="inlineStr">
@@ -2334,18 +2408,18 @@
           <t>Envio de presupuesto</t>
         </is>
       </c>
-      <c r="D45" s="1" t="inlineStr"/>
+      <c r="D45" s="3" t="inlineStr"/>
       <c r="E45" s="1" t="inlineStr">
         <is>
           <t>€1.00</t>
         </is>
       </c>
-      <c r="F45" s="1" t="n">
+      <c r="F45" s="2" t="n">
         <v>1</v>
       </c>
       <c r="G45" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 01:35:58</t>
+          <t>2026-05-26 10:03:09</t>
         </is>
       </c>
       <c r="H45" s="1" t="inlineStr">
@@ -2370,18 +2444,18 @@
           <t>Negociacion</t>
         </is>
       </c>
-      <c r="D46" s="1" t="inlineStr"/>
+      <c r="D46" s="3" t="inlineStr"/>
       <c r="E46" s="1" t="inlineStr">
         <is>
           <t>€0.00</t>
         </is>
       </c>
-      <c r="F46" s="1" t="n">
+      <c r="F46" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G46" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 01:35:58</t>
+          <t>2026-05-26 10:03:09</t>
         </is>
       </c>
       <c r="H46" s="1" t="inlineStr">
@@ -2406,18 +2480,18 @@
           <t>Oportunidad de valor</t>
         </is>
       </c>
-      <c r="D47" s="1" t="inlineStr"/>
+      <c r="D47" s="3" t="inlineStr"/>
       <c r="E47" s="1" t="inlineStr">
         <is>
           <t>€0.00</t>
         </is>
       </c>
-      <c r="F47" s="1" t="n">
+      <c r="F47" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G47" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 01:35:58</t>
+          <t>2026-05-26 10:03:09</t>
         </is>
       </c>
       <c r="H47" s="1" t="inlineStr">
@@ -2442,18 +2516,18 @@
           <t>Por confirmar / Sin respuesta</t>
         </is>
       </c>
-      <c r="D48" s="1" t="inlineStr"/>
+      <c r="D48" s="3" t="inlineStr"/>
       <c r="E48" s="1" t="inlineStr">
         <is>
           <t>€0.00</t>
         </is>
       </c>
-      <c r="F48" s="1" t="n">
+      <c r="F48" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G48" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 01:35:58</t>
+          <t>2026-05-26 10:03:09</t>
         </is>
       </c>
       <c r="H48" s="1" t="inlineStr">
@@ -2478,18 +2552,18 @@
           <t>Proceso de compras</t>
         </is>
       </c>
-      <c r="D49" s="1" t="inlineStr"/>
+      <c r="D49" s="3" t="inlineStr"/>
       <c r="E49" s="1" t="inlineStr">
         <is>
           <t>€0.00</t>
         </is>
       </c>
-      <c r="F49" s="1" t="n">
+      <c r="F49" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G49" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 01:35:58</t>
+          <t>2026-05-26 10:03:09</t>
         </is>
       </c>
       <c r="H49" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Remove total column from stage txt export
</commit_message>
<xml_diff>
--- a/ferniq_oportunidad_scraper/resultado_etapa_ferniq.xlsx
+++ b/ferniq_oportunidad_scraper/resultado_etapa_ferniq.xlsx
@@ -847,7 +847,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Ismael Serrano</t>
+          <t>Javier Barcelo</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -863,15 +863,15 @@
       <c r="D2" s="3" t="inlineStr"/>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>€0.00</t>
+          <t>€3,000.00</t>
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="G2" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 10:03:09</t>
+          <t>2026-05-26 10:59:25</t>
         </is>
       </c>
       <c r="H2" s="1" t="inlineStr">
@@ -883,7 +883,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Ismael Serrano</t>
+          <t>Javier Barcelo</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -907,7 +907,7 @@
       </c>
       <c r="G3" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 10:03:09</t>
+          <t>2026-05-26 10:59:25</t>
         </is>
       </c>
       <c r="H3" s="1" t="inlineStr">
@@ -919,7 +919,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>Ismael Serrano</t>
+          <t>Javier Barcelo</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
@@ -943,7 +943,7 @@
       </c>
       <c r="G4" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 10:03:09</t>
+          <t>2026-05-26 10:59:25</t>
         </is>
       </c>
       <c r="H4" s="1" t="inlineStr">
@@ -955,7 +955,7 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>Ismael Serrano</t>
+          <t>Javier Barcelo</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
@@ -979,7 +979,7 @@
       </c>
       <c r="G5" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 10:03:09</t>
+          <t>2026-05-26 10:59:25</t>
         </is>
       </c>
       <c r="H5" s="1" t="inlineStr">
@@ -991,7 +991,7 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>Ismael Serrano</t>
+          <t>Javier Barcelo</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
@@ -1015,7 +1015,7 @@
       </c>
       <c r="G6" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 10:03:09</t>
+          <t>2026-05-26 10:59:25</t>
         </is>
       </c>
       <c r="H6" s="1" t="inlineStr">
@@ -1027,7 +1027,7 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>Ismael Serrano</t>
+          <t>Javier Barcelo</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr">
@@ -1051,7 +1051,7 @@
       </c>
       <c r="G7" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 10:03:09</t>
+          <t>2026-05-26 10:59:25</t>
         </is>
       </c>
       <c r="H7" s="1" t="inlineStr">
@@ -1063,7 +1063,7 @@
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>Ismael Serrano</t>
+          <t>Javier Barcelo</t>
         </is>
       </c>
       <c r="B8" s="1" t="inlineStr">
@@ -1087,7 +1087,7 @@
       </c>
       <c r="G8" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 10:03:09</t>
+          <t>2026-05-26 10:59:25</t>
         </is>
       </c>
       <c r="H8" s="1" t="inlineStr">
@@ -1099,7 +1099,7 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>Ismael Serrano</t>
+          <t>Javier Barcelo</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
@@ -1115,15 +1115,15 @@
       <c r="D9" s="3" t="inlineStr"/>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>€7,500.00</t>
+          <t>€9,000.00</t>
         </is>
       </c>
       <c r="F9" s="2" t="n">
-        <v>7500</v>
+        <v>9000</v>
       </c>
       <c r="G9" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 10:03:09</t>
+          <t>2026-05-26 10:59:25</t>
         </is>
       </c>
       <c r="H9" s="1" t="inlineStr">
@@ -1135,7 +1135,7 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>Javier Barcelo</t>
+          <t>Ismael Serrano</t>
         </is>
       </c>
       <c r="B10" s="1" t="inlineStr">
@@ -1151,15 +1151,15 @@
       <c r="D10" s="3" t="inlineStr"/>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>€3,000.00</t>
+          <t>€0.00</t>
         </is>
       </c>
       <c r="F10" s="2" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="G10" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 10:03:09</t>
+          <t>2026-05-26 10:59:25</t>
         </is>
       </c>
       <c r="H10" s="1" t="inlineStr">
@@ -1171,7 +1171,7 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>Javier Barcelo</t>
+          <t>Ismael Serrano</t>
         </is>
       </c>
       <c r="B11" s="1" t="inlineStr">
@@ -1195,7 +1195,7 @@
       </c>
       <c r="G11" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 10:03:09</t>
+          <t>2026-05-26 10:59:25</t>
         </is>
       </c>
       <c r="H11" s="1" t="inlineStr">
@@ -1207,7 +1207,7 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>Javier Barcelo</t>
+          <t>Ismael Serrano</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
@@ -1231,7 +1231,7 @@
       </c>
       <c r="G12" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 10:03:09</t>
+          <t>2026-05-26 10:59:25</t>
         </is>
       </c>
       <c r="H12" s="1" t="inlineStr">
@@ -1243,7 +1243,7 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>Javier Barcelo</t>
+          <t>Ismael Serrano</t>
         </is>
       </c>
       <c r="B13" s="1" t="inlineStr">
@@ -1267,7 +1267,7 @@
       </c>
       <c r="G13" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 10:03:09</t>
+          <t>2026-05-26 10:59:25</t>
         </is>
       </c>
       <c r="H13" s="1" t="inlineStr">
@@ -1279,7 +1279,7 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>Javier Barcelo</t>
+          <t>Ismael Serrano</t>
         </is>
       </c>
       <c r="B14" s="1" t="inlineStr">
@@ -1303,7 +1303,7 @@
       </c>
       <c r="G14" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 10:03:09</t>
+          <t>2026-05-26 10:59:25</t>
         </is>
       </c>
       <c r="H14" s="1" t="inlineStr">
@@ -1315,7 +1315,7 @@
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>Javier Barcelo</t>
+          <t>Ismael Serrano</t>
         </is>
       </c>
       <c r="B15" s="1" t="inlineStr">
@@ -1339,7 +1339,7 @@
       </c>
       <c r="G15" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 10:03:09</t>
+          <t>2026-05-26 10:59:25</t>
         </is>
       </c>
       <c r="H15" s="1" t="inlineStr">
@@ -1351,7 +1351,7 @@
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>Javier Barcelo</t>
+          <t>Ismael Serrano</t>
         </is>
       </c>
       <c r="B16" s="1" t="inlineStr">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="G16" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 10:03:09</t>
+          <t>2026-05-26 10:59:25</t>
         </is>
       </c>
       <c r="H16" s="1" t="inlineStr">
@@ -1387,7 +1387,7 @@
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>Javier Barcelo</t>
+          <t>Ismael Serrano</t>
         </is>
       </c>
       <c r="B17" s="1" t="inlineStr">
@@ -1403,15 +1403,15 @@
       <c r="D17" s="3" t="inlineStr"/>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>€9,000.00</t>
+          <t>€7,500.00</t>
         </is>
       </c>
       <c r="F17" s="2" t="n">
-        <v>9000</v>
+        <v>7500</v>
       </c>
       <c r="G17" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 10:03:09</t>
+          <t>2026-05-26 10:59:25</t>
         </is>
       </c>
       <c r="H17" s="1" t="inlineStr">
@@ -1447,7 +1447,7 @@
       </c>
       <c r="G18" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 10:03:09</t>
+          <t>2026-05-26 10:59:25</t>
         </is>
       </c>
       <c r="H18" s="1" t="inlineStr">
@@ -1483,7 +1483,7 @@
       </c>
       <c r="G19" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 10:03:09</t>
+          <t>2026-05-26 10:59:25</t>
         </is>
       </c>
       <c r="H19" s="1" t="inlineStr">
@@ -1519,7 +1519,7 @@
       </c>
       <c r="G20" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 10:03:09</t>
+          <t>2026-05-26 10:59:25</t>
         </is>
       </c>
       <c r="H20" s="1" t="inlineStr">
@@ -1555,7 +1555,7 @@
       </c>
       <c r="G21" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 10:03:09</t>
+          <t>2026-05-26 10:59:25</t>
         </is>
       </c>
       <c r="H21" s="1" t="inlineStr">
@@ -1591,7 +1591,7 @@
       </c>
       <c r="G22" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 10:03:09</t>
+          <t>2026-05-26 10:59:25</t>
         </is>
       </c>
       <c r="H22" s="1" t="inlineStr">
@@ -1627,7 +1627,7 @@
       </c>
       <c r="G23" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 10:03:09</t>
+          <t>2026-05-26 10:59:25</t>
         </is>
       </c>
       <c r="H23" s="1" t="inlineStr">
@@ -1663,7 +1663,7 @@
       </c>
       <c r="G24" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 10:03:09</t>
+          <t>2026-05-26 10:59:25</t>
         </is>
       </c>
       <c r="H24" s="1" t="inlineStr">
@@ -1699,7 +1699,7 @@
       </c>
       <c r="G25" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 10:03:09</t>
+          <t>2026-05-26 10:59:25</t>
         </is>
       </c>
       <c r="H25" s="1" t="inlineStr">
@@ -1735,7 +1735,7 @@
       </c>
       <c r="G26" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 10:03:09</t>
+          <t>2026-05-26 10:59:25</t>
         </is>
       </c>
       <c r="H26" s="1" t="inlineStr">
@@ -1771,7 +1771,7 @@
       </c>
       <c r="G27" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 10:03:09</t>
+          <t>2026-05-26 10:59:25</t>
         </is>
       </c>
       <c r="H27" s="1" t="inlineStr">
@@ -1807,7 +1807,7 @@
       </c>
       <c r="G28" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 10:03:09</t>
+          <t>2026-05-26 10:59:25</t>
         </is>
       </c>
       <c r="H28" s="1" t="inlineStr">
@@ -1843,7 +1843,7 @@
       </c>
       <c r="G29" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 10:03:09</t>
+          <t>2026-05-26 10:59:25</t>
         </is>
       </c>
       <c r="H29" s="1" t="inlineStr">
@@ -1879,7 +1879,7 @@
       </c>
       <c r="G30" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 10:03:09</t>
+          <t>2026-05-26 10:59:25</t>
         </is>
       </c>
       <c r="H30" s="1" t="inlineStr">
@@ -1915,7 +1915,7 @@
       </c>
       <c r="G31" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 10:03:09</t>
+          <t>2026-05-26 10:59:25</t>
         </is>
       </c>
       <c r="H31" s="1" t="inlineStr">
@@ -1951,7 +1951,7 @@
       </c>
       <c r="G32" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 10:03:09</t>
+          <t>2026-05-26 10:59:25</t>
         </is>
       </c>
       <c r="H32" s="1" t="inlineStr">
@@ -1987,7 +1987,7 @@
       </c>
       <c r="G33" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 10:03:09</t>
+          <t>2026-05-26 10:59:25</t>
         </is>
       </c>
       <c r="H33" s="1" t="inlineStr">
@@ -2023,7 +2023,7 @@
       </c>
       <c r="G34" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 10:03:09</t>
+          <t>2026-05-26 10:59:25</t>
         </is>
       </c>
       <c r="H34" s="1" t="inlineStr">
@@ -2059,7 +2059,7 @@
       </c>
       <c r="G35" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 10:03:09</t>
+          <t>2026-05-26 10:59:25</t>
         </is>
       </c>
       <c r="H35" s="1" t="inlineStr">
@@ -2095,7 +2095,7 @@
       </c>
       <c r="G36" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 10:03:09</t>
+          <t>2026-05-26 10:59:25</t>
         </is>
       </c>
       <c r="H36" s="1" t="inlineStr">
@@ -2131,7 +2131,7 @@
       </c>
       <c r="G37" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 10:03:09</t>
+          <t>2026-05-26 10:59:25</t>
         </is>
       </c>
       <c r="H37" s="1" t="inlineStr">
@@ -2167,7 +2167,7 @@
       </c>
       <c r="G38" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 10:03:09</t>
+          <t>2026-05-26 10:59:25</t>
         </is>
       </c>
       <c r="H38" s="1" t="inlineStr">
@@ -2203,7 +2203,7 @@
       </c>
       <c r="G39" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 10:03:09</t>
+          <t>2026-05-26 10:59:25</t>
         </is>
       </c>
       <c r="H39" s="1" t="inlineStr">
@@ -2239,7 +2239,7 @@
       </c>
       <c r="G40" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 10:03:09</t>
+          <t>2026-05-26 10:59:25</t>
         </is>
       </c>
       <c r="H40" s="1" t="inlineStr">
@@ -2275,7 +2275,7 @@
       </c>
       <c r="G41" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 10:03:09</t>
+          <t>2026-05-26 10:59:25</t>
         </is>
       </c>
       <c r="H41" s="1" t="inlineStr">
@@ -2311,7 +2311,7 @@
       </c>
       <c r="G42" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 10:03:09</t>
+          <t>2026-05-26 10:59:25</t>
         </is>
       </c>
       <c r="H42" s="1" t="inlineStr">
@@ -2347,7 +2347,7 @@
       </c>
       <c r="G43" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 10:03:09</t>
+          <t>2026-05-26 10:59:25</t>
         </is>
       </c>
       <c r="H43" s="1" t="inlineStr">
@@ -2383,7 +2383,7 @@
       </c>
       <c r="G44" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 10:03:09</t>
+          <t>2026-05-26 10:59:25</t>
         </is>
       </c>
       <c r="H44" s="1" t="inlineStr">
@@ -2419,7 +2419,7 @@
       </c>
       <c r="G45" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 10:03:09</t>
+          <t>2026-05-26 10:59:25</t>
         </is>
       </c>
       <c r="H45" s="1" t="inlineStr">
@@ -2455,7 +2455,7 @@
       </c>
       <c r="G46" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 10:03:09</t>
+          <t>2026-05-26 10:59:25</t>
         </is>
       </c>
       <c r="H46" s="1" t="inlineStr">
@@ -2491,7 +2491,7 @@
       </c>
       <c r="G47" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 10:03:09</t>
+          <t>2026-05-26 10:59:25</t>
         </is>
       </c>
       <c r="H47" s="1" t="inlineStr">
@@ -2527,7 +2527,7 @@
       </c>
       <c r="G48" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 10:03:09</t>
+          <t>2026-05-26 10:59:25</t>
         </is>
       </c>
       <c r="H48" s="1" t="inlineStr">
@@ -2563,7 +2563,7 @@
       </c>
       <c r="G49" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 10:03:09</t>
+          <t>2026-05-26 10:59:25</t>
         </is>
       </c>
       <c r="H49" s="1" t="inlineStr">

</xml_diff>